<commit_message>
integrated ht as py files
</commit_message>
<xml_diff>
--- a/01_data/dictionary/groups_dictionary_cl.xlsx
+++ b/01_data/dictionary/groups_dictionary_cl.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maxweiland/Desktop/SEDS/Master_Thesis/01_data/dictionary/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EDC404D-A424-C744-B055-8675726391E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C51ECFE2-312D-7542-9C38-19FEB8106AFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1000" yWindow="920" windowWidth="28240" windowHeight="17240" xr2:uid="{1B9E51CD-3202-A34B-B6E9-3062A04AABBD}"/>
   </bookViews>
@@ -187,9 +187,6 @@
     <t>homeowners</t>
   </si>
   <si>
-    <t>homeless pepole</t>
-  </si>
-  <si>
     <t>country dwellers</t>
   </si>
   <si>
@@ -748,9 +745,6 @@
     <t>accountants</t>
   </si>
   <si>
-    <t xml:space="preserve"> truck drivers</t>
-  </si>
-  <si>
     <t xml:space="preserve"> waiters</t>
   </si>
   <si>
@@ -1184,6 +1178,12 @@
   </si>
   <si>
     <t>asylum seekers</t>
+  </si>
+  <si>
+    <t>truck drivers</t>
+  </si>
+  <si>
+    <t>homeless people</t>
   </si>
 </sst>
 </file>
@@ -1688,7 +1688,7 @@
     <col min="40" max="40" width="24.5" customWidth="1"/>
     <col min="41" max="42" width="18.5" customWidth="1"/>
     <col min="43" max="43" width="20.1640625" customWidth="1"/>
-    <col min="45" max="45" width="12" customWidth="1"/>
+    <col min="45" max="45" width="16.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:50" x14ac:dyDescent="0.2">
@@ -1696,16 +1696,16 @@
         <v>13</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>22</v>
@@ -1714,52 +1714,52 @@
         <v>21</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>14</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>318</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>319</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>320</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>9</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="Q1" s="1" t="s">
         <v>18</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="S1" s="1" t="s">
+        <v>325</v>
+      </c>
+      <c r="T1" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="T1" s="1" t="s">
-        <v>329</v>
-      </c>
       <c r="U1" s="1" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="X1" s="1" t="s">
         <v>10</v>
@@ -1771,25 +1771,25 @@
         <v>5</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="AB1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="AD1" s="1" t="s">
         <v>17</v>
       </c>
       <c r="AE1" s="1" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="AF1" s="1" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="AG1" s="1" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="AH1" s="1" t="s">
         <v>19</v>
@@ -1801,13 +1801,13 @@
         <v>2</v>
       </c>
       <c r="AK1" s="1" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="AL1" s="1" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="AM1" s="1" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="AN1" s="1" t="s">
         <v>1</v>
@@ -1819,7 +1819,7 @@
         <v>20</v>
       </c>
       <c r="AQ1" s="1" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="AR1" s="1" t="s">
         <v>16</v>
@@ -1835,37 +1835,37 @@
     </row>
     <row r="2" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A2" s="8" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>38</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="K2" s="8" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="L2" s="2" t="s">
         <v>31</v>
@@ -1877,10 +1877,10 @@
         <v>26</v>
       </c>
       <c r="O2" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="P2" s="10" t="s">
-        <v>47</v>
+        <v>379</v>
       </c>
       <c r="Q2" s="10" t="s">
         <v>46</v>
@@ -1889,19 +1889,19 @@
         <v>32</v>
       </c>
       <c r="S2" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="T2" s="11" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="U2" s="2" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="V2" s="10" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="W2" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="X2" s="5" t="s">
         <v>36</v>
@@ -1913,28 +1913,28 @@
         <v>28</v>
       </c>
       <c r="AA2" s="2" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="AB2" s="2" t="s">
         <v>27</v>
       </c>
       <c r="AC2" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="AD2" s="2" t="s">
         <v>40</v>
       </c>
       <c r="AE2" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AF2" s="2" t="s">
         <v>41</v>
       </c>
       <c r="AG2" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AH2" s="10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="AI2" s="12" t="s">
         <v>23</v>
@@ -1943,13 +1943,13 @@
         <v>25</v>
       </c>
       <c r="AK2" s="2" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="AL2" s="2" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="AM2" s="2" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="AN2" s="2" t="s">
         <v>24</v>
@@ -1958,16 +1958,16 @@
         <v>29</v>
       </c>
       <c r="AP2" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="AQ2" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="AR2" s="2" t="s">
         <v>16</v>
       </c>
       <c r="AS2" s="2" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="AT2" s="2"/>
       <c r="AU2" s="2"/>
@@ -1980,130 +1980,130 @@
         <v>37</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="I3" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="K3" s="9" t="s">
+        <v>350</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="O3" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="P3" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="Q3" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="R3" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="S3" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="T3" s="10" t="s">
+        <v>352</v>
+      </c>
+      <c r="U3" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="J3" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="K3" s="9" t="s">
-        <v>352</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="M3" s="3" t="s">
+      <c r="V3" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="W3" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="X3" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="N3" s="3" t="s">
-        <v>322</v>
-      </c>
-      <c r="O3" s="11" t="s">
-        <v>113</v>
-      </c>
-      <c r="P3" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="Q3" s="11" t="s">
-        <v>77</v>
-      </c>
-      <c r="R3" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="S3" s="3" t="s">
-        <v>328</v>
-      </c>
-      <c r="T3" s="10" t="s">
-        <v>354</v>
-      </c>
-      <c r="U3" s="3" t="s">
+      <c r="Y3" s="3" t="s">
+        <v>330</v>
+      </c>
+      <c r="Z3" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="AA3" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="AB3" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="AC3" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="AD3" s="3" t="s">
         <v>71</v>
-      </c>
-      <c r="V3" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="W3" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="X3" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="Y3" s="3" t="s">
-        <v>332</v>
-      </c>
-      <c r="Z3" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="AA3" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="AB3" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="AC3" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="AD3" s="3" t="s">
-        <v>72</v>
       </c>
       <c r="AE3" s="3"/>
       <c r="AF3" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="AG3" s="6" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AH3" s="11" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AI3" s="13"/>
       <c r="AJ3" s="2" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="AK3" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="AL3" s="3"/>
       <c r="AM3" s="3" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="AN3" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AO3" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="AP3" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AQ3" s="3" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="AR3" s="3" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="AS3" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AT3" s="3"/>
       <c r="AU3" s="3"/>
@@ -2114,120 +2114,120 @@
     <row r="4" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A4" s="8"/>
       <c r="B4" s="2" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="E4" s="2"/>
       <c r="F4" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="K4" s="2"/>
       <c r="L4" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="N4" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="O4" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="P4" s="10" t="s">
+        <v>351</v>
+      </c>
+      <c r="Q4" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="R4" s="5" t="s">
         <v>91</v>
-      </c>
-      <c r="M4" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="N4" s="2" t="s">
-        <v>323</v>
-      </c>
-      <c r="O4" s="10" t="s">
-        <v>137</v>
-      </c>
-      <c r="P4" s="10" t="s">
-        <v>353</v>
-      </c>
-      <c r="Q4" s="10" t="s">
-        <v>104</v>
-      </c>
-      <c r="R4" s="5" t="s">
-        <v>92</v>
       </c>
       <c r="S4" s="2"/>
       <c r="T4" s="11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="U4" s="2" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="V4" s="10" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="W4" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="X4" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="Y4" s="2"/>
       <c r="Z4" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AA4" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="AB4" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="AC4" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="AD4" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="AE4" s="2"/>
       <c r="AF4" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="AG4" s="5" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="AH4" s="10" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="AI4" s="12"/>
       <c r="AJ4" s="3" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="AK4" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="AL4" s="2"/>
       <c r="AM4" s="2" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="AN4" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="AO4" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AP4" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="AQ4" s="2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="AR4" s="2"/>
       <c r="AS4" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="AT4" s="2"/>
       <c r="AU4" s="2"/>
@@ -2238,116 +2238,116 @@
     <row r="5" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A5" s="9"/>
       <c r="B5" s="3" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
       <c r="F5" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K5" s="3"/>
       <c r="L5" s="3" t="s">
         <v>33</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="N5" s="3"/>
       <c r="O5" s="11" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="P5" s="11" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q5" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="R5" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="S5" s="3"/>
       <c r="T5" s="10" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="U5" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="V5" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="W5" s="3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="X5" s="6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="Y5" s="3"/>
       <c r="Z5" s="11" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="AA5" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AB5" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AC5" s="3" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="AD5" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="AE5" s="3"/>
       <c r="AF5" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="AG5" s="6" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="AH5" s="11" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="AI5" s="13"/>
       <c r="AJ5" s="2" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="AK5" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="AL5" s="3"/>
       <c r="AM5" s="3" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="AN5" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="AO5" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="AP5" s="6" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AQ5" s="2" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="AR5" s="3"/>
       <c r="AS5" s="3" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="AT5" s="3"/>
       <c r="AU5" s="3"/>
@@ -2359,21 +2359,21 @@
       <c r="A6" s="8"/>
       <c r="B6" s="2"/>
       <c r="C6" s="10" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
@@ -2381,83 +2381,83 @@
         <v>8</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="N6" s="2"/>
       <c r="O6" s="10" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="P6" s="2"/>
       <c r="Q6" s="10" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="S6" s="2"/>
       <c r="T6" s="11" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="U6" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="V6" s="10" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W6" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="X6" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="Y6" s="2"/>
       <c r="Z6" s="2"/>
       <c r="AA6" s="2" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="AB6" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="AC6" s="2" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="AD6" s="3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="AE6" s="2"/>
       <c r="AF6" s="2" t="s">
         <v>42</v>
       </c>
       <c r="AG6" s="5" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="AH6" s="10" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="AI6" s="12"/>
       <c r="AJ6" s="3" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="AK6" s="2" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="AL6" s="2"/>
       <c r="AM6" s="2" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="AN6" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="AO6" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AP6" s="2"/>
       <c r="AQ6" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="AR6" s="2"/>
       <c r="AS6" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="AT6" s="2"/>
       <c r="AU6" s="2"/>
@@ -2469,21 +2469,21 @@
       <c r="A7" s="9"/>
       <c r="B7" s="3"/>
       <c r="C7" s="11" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
       <c r="F7" s="3" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
@@ -2491,15 +2491,15 @@
         <v>34</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="N7" s="3"/>
       <c r="O7" s="11" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="P7" s="3"/>
       <c r="Q7" s="11" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R7" s="6" t="s">
         <v>7</v>
@@ -2507,44 +2507,44 @@
       <c r="S7" s="3"/>
       <c r="T7" s="10"/>
       <c r="U7" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="V7" s="11" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="W7" s="3" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="X7" s="6" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="Y7" s="3"/>
       <c r="Z7" s="3"/>
       <c r="AA7" s="3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="AB7" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AC7" s="3" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="AD7" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AE7" s="3"/>
       <c r="AF7" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="AG7" s="6" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="AH7" s="11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="AI7" s="13"/>
       <c r="AJ7" s="2" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="AK7" s="3" t="s">
         <v>30</v>
@@ -2552,18 +2552,18 @@
       <c r="AL7" s="3"/>
       <c r="AM7" s="3"/>
       <c r="AN7" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="AO7" s="3" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AP7" s="3"/>
       <c r="AQ7" s="2" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="AR7" s="3"/>
       <c r="AS7" s="3" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="AT7" s="3"/>
       <c r="AU7" s="3"/>
@@ -2578,90 +2578,90 @@
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
       <c r="F8" s="2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="H8" s="2"/>
       <c r="I8" s="2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
       <c r="L8" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="N8" s="2"/>
       <c r="O8" s="10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="P8" s="2"/>
       <c r="Q8" s="10" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="R8" s="5" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="S8" s="2"/>
       <c r="T8" s="11"/>
       <c r="U8" s="2" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V8" s="10" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="W8" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="X8" s="5" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="Y8" s="2"/>
       <c r="Z8" s="2"/>
       <c r="AA8" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AB8" s="2" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="AC8" s="2" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="AD8" s="3" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="AE8" s="2"/>
       <c r="AF8" s="2" t="s">
         <v>44</v>
       </c>
       <c r="AG8" s="5" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="AH8" s="10" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AI8" s="12"/>
       <c r="AJ8" s="3" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="AK8" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="AL8" s="2"/>
       <c r="AM8" s="2"/>
       <c r="AN8" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="AO8" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AP8" s="2"/>
       <c r="AQ8" s="3" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="AR8" s="2"/>
       <c r="AS8" s="2"/>
@@ -2679,81 +2679,81 @@
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
       <c r="G9" s="3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="H9" s="3"/>
       <c r="I9" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
       <c r="L9" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="N9" s="3"/>
       <c r="O9" s="11" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="P9" s="3"/>
       <c r="Q9" s="11" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="R9" s="13"/>
       <c r="S9" s="3"/>
       <c r="T9" s="10"/>
       <c r="U9" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="V9" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="W9" s="3" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="X9" s="3"/>
       <c r="Y9" s="3"/>
       <c r="Z9" s="3"/>
       <c r="AA9" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AB9" s="3" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="AC9" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="AD9" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="AE9" s="3"/>
       <c r="AF9" s="2" t="s">
         <v>45</v>
       </c>
       <c r="AG9" s="6" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="AH9" s="11" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="AI9" s="13"/>
       <c r="AJ9" s="3" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="AK9" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="AL9" s="3"/>
       <c r="AM9" s="3"/>
       <c r="AN9" s="3"/>
       <c r="AO9" s="3" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="AP9" s="3"/>
       <c r="AQ9" s="2" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="AR9" s="3"/>
       <c r="AS9" s="3"/>
@@ -2771,21 +2771,21 @@
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
       <c r="G10" s="2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
       <c r="L10" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="N10" s="2"/>
       <c r="O10" s="10" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="P10" s="2"/>
       <c r="Q10" s="10"/>
@@ -2793,51 +2793,51 @@
       <c r="S10" s="2"/>
       <c r="T10" s="11"/>
       <c r="U10" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="V10" s="10" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="W10" s="2" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="X10" s="2"/>
       <c r="Y10" s="2"/>
       <c r="Z10" s="2"/>
       <c r="AA10" s="2" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="AB10" s="2" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="AC10" s="2"/>
       <c r="AD10" s="3" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="AE10" s="2"/>
       <c r="AF10" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="AG10" s="5" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="AH10" s="10" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="AI10" s="12"/>
       <c r="AJ10" s="2" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="AK10" s="2"/>
       <c r="AL10" s="2"/>
       <c r="AM10" s="2"/>
       <c r="AN10" s="2"/>
       <c r="AO10" s="2" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AP10" s="2"/>
       <c r="AQ10" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="AR10" s="2"/>
       <c r="AS10" s="2"/>
@@ -2855,19 +2855,19 @@
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
       <c r="G11" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
       <c r="L11" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="M11" s="2"/>
       <c r="N11" s="3"/>
       <c r="O11" s="11" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="P11" s="3"/>
       <c r="Q11" s="3"/>
@@ -2875,47 +2875,47 @@
       <c r="S11" s="3"/>
       <c r="T11" s="3"/>
       <c r="U11" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="V11" s="11" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="W11" s="3" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="X11" s="3"/>
       <c r="Y11" s="3"/>
       <c r="Z11" s="3"/>
       <c r="AA11" s="3" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="AB11" s="3"/>
       <c r="AC11" s="3"/>
       <c r="AD11" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="AE11" s="3"/>
       <c r="AF11" s="3" t="s">
         <v>43</v>
       </c>
       <c r="AG11" s="6" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="AH11" s="3"/>
       <c r="AI11" s="3"/>
       <c r="AJ11" s="2" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="AK11" s="3"/>
       <c r="AL11" s="3"/>
       <c r="AM11" s="3"/>
       <c r="AN11" s="3"/>
       <c r="AO11" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="AP11" s="3"/>
       <c r="AQ11" s="3" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="AR11" s="3"/>
       <c r="AS11" s="3"/>
@@ -2933,19 +2933,19 @@
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
       <c r="G12" s="2" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="M12" s="2"/>
       <c r="N12" s="2"/>
       <c r="O12" s="10" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="P12" s="2"/>
       <c r="Q12" s="2"/>
@@ -2953,29 +2953,29 @@
       <c r="S12" s="2"/>
       <c r="T12" s="2"/>
       <c r="U12" s="2" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="V12" s="10" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="W12" s="2" t="s">
-        <v>234</v>
+        <v>378</v>
       </c>
       <c r="X12" s="2"/>
       <c r="Y12" s="2"/>
       <c r="Z12" s="2"/>
       <c r="AA12" s="2" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="AB12" s="2"/>
       <c r="AC12" s="2"/>
       <c r="AD12" s="3" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="AE12" s="2"/>
       <c r="AF12" s="2"/>
       <c r="AG12" s="5" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="AH12" s="2"/>
       <c r="AI12" s="2"/>
@@ -2985,11 +2985,11 @@
       <c r="AM12" s="2"/>
       <c r="AN12" s="2"/>
       <c r="AO12" s="2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AP12" s="2"/>
       <c r="AQ12" s="2" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="AR12" s="2"/>
       <c r="AS12" s="2"/>
@@ -3007,14 +3007,14 @@
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
       <c r="G13" s="3" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
       <c r="J13" s="3"/>
       <c r="K13" s="3"/>
       <c r="L13" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="M13" s="3"/>
       <c r="N13" s="3"/>
@@ -3025,24 +3025,24 @@
       <c r="S13" s="3"/>
       <c r="T13" s="3"/>
       <c r="U13" s="3" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="V13" s="11" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="W13" s="3" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="X13" s="3"/>
       <c r="Y13" s="3"/>
       <c r="Z13" s="3"/>
       <c r="AA13" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="AB13" s="3"/>
       <c r="AC13" s="3"/>
       <c r="AD13" s="3" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="AE13" s="3"/>
       <c r="AF13" s="3"/>
@@ -3055,11 +3055,11 @@
       <c r="AM13" s="3"/>
       <c r="AN13" s="3"/>
       <c r="AO13" s="3" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="AP13" s="3"/>
       <c r="AQ13" s="3" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="AR13" s="3"/>
       <c r="AS13" s="3"/>
@@ -3091,13 +3091,13 @@
       <c r="S14" s="2"/>
       <c r="T14" s="2"/>
       <c r="U14" s="2" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="V14" s="10" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="W14" s="2" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="X14" s="2"/>
       <c r="Y14" s="2"/>
@@ -3119,7 +3119,7 @@
       <c r="AO14" s="2"/>
       <c r="AP14" s="2"/>
       <c r="AQ14" s="2" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="AR14" s="2"/>
       <c r="AS14" s="2"/>
@@ -3152,10 +3152,10 @@
       <c r="T15" s="3"/>
       <c r="U15" s="3"/>
       <c r="V15" s="11" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="W15" s="3" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="X15" s="3"/>
       <c r="Y15" s="3"/>
@@ -3177,7 +3177,7 @@
       <c r="AO15" s="3"/>
       <c r="AP15" s="3"/>
       <c r="AQ15" s="2" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="AR15" s="3"/>
       <c r="AS15" s="3"/>
@@ -3210,10 +3210,10 @@
       <c r="T16" s="2"/>
       <c r="U16" s="2"/>
       <c r="V16" s="10" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="W16" s="2" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="X16" s="2"/>
       <c r="Y16" s="2"/>
@@ -3235,7 +3235,7 @@
       <c r="AO16" s="2"/>
       <c r="AP16" s="2"/>
       <c r="AQ16" s="3" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="AR16" s="2"/>
       <c r="AS16" s="2"/>
@@ -3268,10 +3268,10 @@
       <c r="T17" s="3"/>
       <c r="U17" s="3"/>
       <c r="V17" s="11" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="W17" s="3" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="X17" s="3"/>
       <c r="Y17" s="3"/>
@@ -3293,7 +3293,7 @@
       <c r="AO17" s="3"/>
       <c r="AP17" s="3"/>
       <c r="AQ17" s="2" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="AR17" s="3"/>
       <c r="AS17" s="3"/>
@@ -3326,10 +3326,10 @@
       <c r="T18" s="2"/>
       <c r="U18" s="2"/>
       <c r="V18" s="10" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="W18" s="2" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="X18" s="2"/>
       <c r="Y18" s="2"/>
@@ -3351,7 +3351,7 @@
       <c r="AO18" s="2"/>
       <c r="AP18" s="2"/>
       <c r="AQ18" s="3" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="AR18" s="2"/>
       <c r="AS18" s="2"/>
@@ -3384,10 +3384,10 @@
       <c r="T19" s="3"/>
       <c r="U19" s="3"/>
       <c r="V19" s="11" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="W19" s="6" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="X19" s="3"/>
       <c r="Y19" s="3"/>
@@ -3409,7 +3409,7 @@
       <c r="AO19" s="3"/>
       <c r="AP19" s="3"/>
       <c r="AQ19" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="AR19" s="3"/>
       <c r="AS19" s="3"/>
@@ -3442,10 +3442,10 @@
       <c r="T20" s="2"/>
       <c r="U20" s="2"/>
       <c r="V20" s="10" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="W20" s="5" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="X20" s="2"/>
       <c r="Y20" s="2"/>
@@ -3498,10 +3498,10 @@
       <c r="T21" s="3"/>
       <c r="U21" s="3"/>
       <c r="V21" s="11" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="W21" s="6" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="X21" s="3"/>
       <c r="Y21" s="3"/>
@@ -3554,10 +3554,10 @@
       <c r="T22" s="2"/>
       <c r="U22" s="2"/>
       <c r="V22" s="10" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="W22" s="5" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="X22" s="2"/>
       <c r="Y22" s="2"/>
@@ -3610,10 +3610,10 @@
       <c r="T23" s="3"/>
       <c r="U23" s="3"/>
       <c r="V23" s="11" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="W23" s="6" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="X23" s="3"/>
       <c r="Y23" s="3"/>
@@ -3667,7 +3667,7 @@
       <c r="U24" s="2"/>
       <c r="V24" s="2"/>
       <c r="W24" s="5" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="X24" s="2"/>
       <c r="Y24" s="2"/>
@@ -3699,22 +3699,22 @@
     </row>
     <row r="25" spans="1:50" x14ac:dyDescent="0.2">
       <c r="W25" s="6" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="26" spans="1:50" x14ac:dyDescent="0.2">
       <c r="W26" s="5" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="27" spans="1:50" x14ac:dyDescent="0.2">
       <c r="W27" s="6" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
     </row>
     <row r="28" spans="1:50" x14ac:dyDescent="0.2">
       <c r="W28" s="5" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
implemented clustering and cluster assessment
</commit_message>
<xml_diff>
--- a/01_data/dictionary/groups_dictionary_cl.xlsx
+++ b/01_data/dictionary/groups_dictionary_cl.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maxweiland/Desktop/SEDS/Master_Thesis/01_data/dictionary/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C51ECFE2-312D-7542-9C38-19FEB8106AFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF29E687-2B57-6E46-AA3D-AB53321ED52F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1000" yWindow="920" windowWidth="28240" windowHeight="17240" xr2:uid="{1B9E51CD-3202-A34B-B6E9-3062A04AABBD}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="380">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="399">
   <si>
     <t>Self-employed</t>
   </si>
@@ -115,9 +115,6 @@
     <t>Crime victims</t>
   </si>
   <si>
-    <t>self-employed</t>
-  </si>
-  <si>
     <t>unemployed</t>
   </si>
   <si>
@@ -382,9 +379,6 @@
     <t xml:space="preserve"> plumbers</t>
   </si>
   <si>
-    <t xml:space="preserve"> carers</t>
-  </si>
-  <si>
     <t>constables</t>
   </si>
   <si>
@@ -733,12 +727,6 @@
     <t xml:space="preserve"> hairdressers</t>
   </si>
   <si>
-    <t>special constables</t>
-  </si>
-  <si>
-    <t>investors</t>
-  </si>
-  <si>
     <t>physically or mentally disabled</t>
   </si>
   <si>
@@ -1184,13 +1172,82 @@
   </si>
   <si>
     <t>homeless people</t>
+  </si>
+  <si>
+    <t>all those paying taxes</t>
+  </si>
+  <si>
+    <t>legislators</t>
+  </si>
+  <si>
+    <t>freelancers</t>
+  </si>
+  <si>
+    <t>self-employed people</t>
+  </si>
+  <si>
+    <t>shoppers</t>
+  </si>
+  <si>
+    <t>persons of mature age</t>
+  </si>
+  <si>
+    <t>grown-ups</t>
+  </si>
+  <si>
+    <t>civil employees</t>
+  </si>
+  <si>
+    <t>purchasers</t>
+  </si>
+  <si>
+    <t>labourers</t>
+  </si>
+  <si>
+    <t>ranchers</t>
+  </si>
+  <si>
+    <t>landlord community</t>
+  </si>
+  <si>
+    <t>those who rent out properties</t>
+  </si>
+  <si>
+    <t>male people</t>
+  </si>
+  <si>
+    <t>men in my constituency</t>
+  </si>
+  <si>
+    <t>ministers</t>
+  </si>
+  <si>
+    <t>elected members of parliaments</t>
+  </si>
+  <si>
+    <t>freelancer community</t>
+  </si>
+  <si>
+    <t>independent contractors</t>
+  </si>
+  <si>
+    <t>taxpayers in our country</t>
+  </si>
+  <si>
+    <t>taxpayers in my constituency</t>
+  </si>
+  <si>
+    <t>female people</t>
+  </si>
+  <si>
+    <t>women in my constituency</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1211,6 +1268,12 @@
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -1300,7 +1363,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1315,6 +1378,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1696,16 +1760,16 @@
         <v>13</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>22</v>
@@ -1714,52 +1778,52 @@
         <v>21</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>14</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>9</v>
       </c>
       <c r="N1" s="1" t="s">
+        <v>315</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="P1" s="1" t="s">
         <v>319</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>322</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>323</v>
       </c>
       <c r="Q1" s="1" t="s">
         <v>18</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="V1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="X1" s="1" t="s">
         <v>10</v>
@@ -1771,25 +1835,25 @@
         <v>5</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="AB1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="AD1" s="1" t="s">
         <v>17</v>
       </c>
       <c r="AE1" s="1" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="AF1" s="1" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="AG1" s="1" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="AH1" s="1" t="s">
         <v>19</v>
@@ -1801,13 +1865,13 @@
         <v>2</v>
       </c>
       <c r="AK1" s="1" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
       <c r="AL1" s="1" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="AM1" s="1" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="AN1" s="1" t="s">
         <v>1</v>
@@ -1819,7 +1883,7 @@
         <v>20</v>
       </c>
       <c r="AQ1" s="1" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="AR1" s="1" t="s">
         <v>16</v>
@@ -1835,139 +1899,139 @@
     </row>
     <row r="2" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A2" s="8" t="s">
+        <v>304</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>338</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>308</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>267</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>342</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="G2" s="2" t="s">
+      <c r="I2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="K2" s="8" t="s">
         <v>345</v>
       </c>
-      <c r="H2" s="2" t="s">
-        <v>312</v>
-      </c>
-      <c r="I2" s="2" t="s">
+      <c r="L2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="O2" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="P2" s="10" t="s">
+        <v>375</v>
+      </c>
+      <c r="Q2" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="R2" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="T2" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="U2" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="V2" s="10" t="s">
+        <v>354</v>
+      </c>
+      <c r="W2" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="X2" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y2" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="J2" s="2" t="s">
-        <v>348</v>
-      </c>
-      <c r="K2" s="8" t="s">
-        <v>349</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="N2" s="2" t="s">
+      <c r="Z2" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA2" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="AB2" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="O2" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="P2" s="10" t="s">
+      <c r="AC2" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="AD2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="AE2" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="AF2" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="AG2" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="AH2" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="AI2" s="12" t="s">
         <v>379</v>
       </c>
-      <c r="Q2" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="R2" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="S2" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="T2" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="U2" s="2" t="s">
-        <v>355</v>
-      </c>
-      <c r="V2" s="10" t="s">
-        <v>358</v>
-      </c>
-      <c r="W2" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="X2" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="Y2" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="Z2" s="10" t="s">
+      <c r="AJ2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="AK2" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="AL2" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="AM2" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="AN2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="AO2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="AA2" s="2" t="s">
-        <v>369</v>
-      </c>
-      <c r="AB2" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="AC2" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="AD2" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="AE2" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="AF2" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="AG2" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="AH2" s="10" t="s">
+      <c r="AP2" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="AI2" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="AJ2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="AK2" s="2" t="s">
-        <v>373</v>
-      </c>
-      <c r="AL2" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="AM2" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="AN2" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="AO2" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="AP2" s="5" t="s">
-        <v>48</v>
-      </c>
       <c r="AQ2" s="3" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="AR2" s="2" t="s">
         <v>16</v>
       </c>
       <c r="AS2" s="2" t="s">
-        <v>374</v>
+        <v>370</v>
       </c>
       <c r="AT2" s="2"/>
       <c r="AU2" s="2"/>
@@ -1977,133 +2041,139 @@
     </row>
     <row r="3" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A3" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="I3" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="K3" s="9" t="s">
+        <v>346</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="O3" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="P3" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="Q3" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="R3" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="S3" s="3" t="s">
+        <v>322</v>
+      </c>
+      <c r="T3" s="10" t="s">
+        <v>348</v>
+      </c>
+      <c r="U3" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="V3" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="W3" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="X3" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="Y3" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="Z3" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="AA3" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="AB3" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="AC3" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="AD3" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="AE3" s="3" t="s">
+        <v>377</v>
+      </c>
+      <c r="AF3" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="AG3" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="AH3" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="AI3" s="13" t="s">
+        <v>378</v>
+      </c>
+      <c r="AJ3" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="AK3" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="AL3" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="AM3" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="AN3" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="K3" s="9" t="s">
-        <v>350</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="M3" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="N3" s="3" t="s">
-        <v>320</v>
-      </c>
-      <c r="O3" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="P3" s="11" t="s">
-        <v>77</v>
-      </c>
-      <c r="Q3" s="11" t="s">
-        <v>76</v>
-      </c>
-      <c r="R3" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="S3" s="3" t="s">
-        <v>326</v>
-      </c>
-      <c r="T3" s="10" t="s">
-        <v>352</v>
-      </c>
-      <c r="U3" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="V3" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="W3" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="X3" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="Y3" s="3" t="s">
-        <v>330</v>
-      </c>
-      <c r="Z3" s="11" t="s">
+      <c r="AO3" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="AA3" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AB3" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="AC3" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="AD3" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="AE3" s="3"/>
-      <c r="AF3" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="AG3" s="6" t="s">
-        <v>207</v>
-      </c>
-      <c r="AH3" s="11" t="s">
+      <c r="AP3" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="AI3" s="13"/>
-      <c r="AJ3" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="AK3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AL3" s="3"/>
-      <c r="AM3" s="3" t="s">
-        <v>335</v>
-      </c>
-      <c r="AN3" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="AO3" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="AP3" s="6" t="s">
-        <v>79</v>
-      </c>
       <c r="AQ3" s="3" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="AR3" s="3" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="AS3" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AT3" s="3"/>
       <c r="AU3" s="3"/>
@@ -2112,122 +2182,140 @@
       <c r="AX3" s="6"/>
     </row>
     <row r="4" spans="1:50" x14ac:dyDescent="0.2">
-      <c r="A4" s="8"/>
+      <c r="A4" s="14" t="s">
+        <v>381</v>
+      </c>
       <c r="B4" s="2" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>310</v>
-      </c>
-      <c r="E4" s="2"/>
+        <v>306</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>380</v>
+      </c>
       <c r="F4" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>346</v>
+        <v>342</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="I4" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="N4" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="O4" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="P4" s="10" t="s">
+        <v>347</v>
+      </c>
+      <c r="Q4" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="R4" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="S4" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="T4" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="U4" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="V4" s="10" t="s">
+        <v>355</v>
+      </c>
+      <c r="W4" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="X4" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="Y4" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="Z4" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="AA4" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="AB4" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="AC4" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="AD4" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="AE4" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="AF4" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="AG4" s="5" t="s">
+        <v>283</v>
+      </c>
+      <c r="AH4" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="AI4" s="12" t="s">
+        <v>393</v>
+      </c>
+      <c r="AJ4" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="AK4" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="AL4" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="AM4" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="AN4" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="M4" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="N4" s="2" t="s">
-        <v>321</v>
-      </c>
-      <c r="O4" s="10" t="s">
-        <v>136</v>
-      </c>
-      <c r="P4" s="10" t="s">
-        <v>351</v>
-      </c>
-      <c r="Q4" s="10" t="s">
-        <v>103</v>
-      </c>
-      <c r="R4" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="S4" s="2"/>
-      <c r="T4" s="11" t="s">
-        <v>113</v>
-      </c>
-      <c r="U4" s="2" t="s">
-        <v>356</v>
-      </c>
-      <c r="V4" s="10" t="s">
-        <v>359</v>
-      </c>
-      <c r="W4" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="X4" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="Y4" s="2"/>
-      <c r="Z4" s="10" t="s">
+      <c r="AO4" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="AA4" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="AB4" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="AC4" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="AD4" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="AE4" s="2"/>
-      <c r="AF4" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="AG4" s="5" t="s">
-        <v>287</v>
-      </c>
-      <c r="AH4" s="10" t="s">
+      <c r="AP4" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="AI4" s="12"/>
-      <c r="AJ4" s="3" t="s">
-        <v>238</v>
-      </c>
-      <c r="AK4" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="AL4" s="2"/>
-      <c r="AM4" s="2" t="s">
-        <v>336</v>
-      </c>
-      <c r="AN4" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="AO4" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="AP4" s="5" t="s">
-        <v>105</v>
-      </c>
       <c r="AQ4" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="AR4" s="2"/>
+        <v>228</v>
+      </c>
+      <c r="AR4" s="2" t="s">
+        <v>397</v>
+      </c>
       <c r="AS4" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="AT4" s="2"/>
       <c r="AU4" s="2"/>
@@ -2236,118 +2324,140 @@
       <c r="AX4" s="5"/>
     </row>
     <row r="5" spans="1:50" x14ac:dyDescent="0.2">
-      <c r="A5" s="9"/>
+      <c r="A5" s="9" t="s">
+        <v>382</v>
+      </c>
       <c r="B5" s="3" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="C5" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>383</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>384</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="I5" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>347</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>314</v>
-      </c>
-      <c r="I5" s="3" t="s">
+      <c r="J5" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>385</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="N5" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="O5" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="P5" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="Q5" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="R5" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="S5" s="3" t="s">
+        <v>388</v>
+      </c>
+      <c r="T5" s="10" t="s">
+        <v>199</v>
+      </c>
+      <c r="U5" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="V5" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="W5" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="X5" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="Y5" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="Z5" s="11" t="s">
+        <v>364</v>
+      </c>
+      <c r="AA5" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="AB5" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="AC5" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="AD5" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="J5" s="3" t="s">
+      <c r="AE5" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="AF5" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="AG5" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="AH5" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="AI5" s="13" t="s">
+        <v>394</v>
+      </c>
+      <c r="AJ5" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="AK5" t="s">
+        <v>329</v>
+      </c>
+      <c r="AL5" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="AM5" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="AN5" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="K5" s="3"/>
-      <c r="L5" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="M5" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="N5" s="3"/>
-      <c r="O5" s="11" t="s">
-        <v>84</v>
-      </c>
-      <c r="P5" s="11" t="s">
+      <c r="AO5" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="AP5" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="Q5" s="11" t="s">
-        <v>127</v>
-      </c>
-      <c r="R5" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="S5" s="3"/>
-      <c r="T5" s="10" t="s">
-        <v>201</v>
-      </c>
-      <c r="U5" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="V5" s="11" t="s">
-        <v>114</v>
-      </c>
-      <c r="W5" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="X5" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="Y5" s="3"/>
-      <c r="Z5" s="11" t="s">
-        <v>368</v>
-      </c>
-      <c r="AA5" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="AB5" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="AC5" s="3" t="s">
-        <v>297</v>
-      </c>
-      <c r="AD5" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="AE5" s="3"/>
-      <c r="AF5" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="AG5" s="6" t="s">
-        <v>288</v>
-      </c>
-      <c r="AH5" s="11" t="s">
-        <v>129</v>
-      </c>
-      <c r="AI5" s="13"/>
-      <c r="AJ5" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="AK5" t="s">
-        <v>333</v>
-      </c>
-      <c r="AL5" s="3"/>
-      <c r="AM5" s="3" t="s">
-        <v>337</v>
-      </c>
-      <c r="AN5" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="AO5" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="AP5" s="6" t="s">
-        <v>130</v>
-      </c>
       <c r="AQ5" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="AR5" s="3"/>
+        <v>251</v>
+      </c>
+      <c r="AR5" s="3" t="s">
+        <v>398</v>
+      </c>
       <c r="AS5" s="3" t="s">
-        <v>375</v>
+        <v>371</v>
       </c>
       <c r="AT5" s="3"/>
       <c r="AU5" s="3"/>
@@ -2359,105 +2469,107 @@
       <c r="A6" s="8"/>
       <c r="B6" s="2"/>
       <c r="C6" s="10" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="J6" s="2"/>
+        <v>145</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>278</v>
+      </c>
       <c r="K6" s="2"/>
       <c r="L6" s="2" t="s">
         <v>8</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="N6" s="2"/>
-      <c r="O6" s="10" t="s">
-        <v>110</v>
+      <c r="O6" s="11" t="s">
+        <v>132</v>
       </c>
       <c r="P6" s="2"/>
       <c r="Q6" s="10" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="S6" s="2"/>
       <c r="T6" s="11" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="U6" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="V6" s="10" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="W6" s="2" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="X6" s="5" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="Y6" s="2"/>
       <c r="Z6" s="2"/>
       <c r="AA6" s="2" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="AB6" s="3" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="AC6" s="2" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="AD6" s="3" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="AE6" s="2"/>
       <c r="AF6" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="AG6" s="5" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="AH6" s="10" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="AI6" s="12"/>
       <c r="AJ6" s="3" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="AK6" s="2" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="AL6" s="2"/>
       <c r="AM6" s="2" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
       <c r="AN6" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="AO6" s="2" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="AP6" s="2"/>
       <c r="AQ6" s="3" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="AR6" s="2"/>
       <c r="AS6" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="AT6" s="2"/>
       <c r="AU6" s="2"/>
@@ -2469,37 +2581,37 @@
       <c r="A7" s="9"/>
       <c r="B7" s="3"/>
       <c r="C7" s="11" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
       <c r="F7" s="3" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
       <c r="L7" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="N7" s="3"/>
-      <c r="O7" s="11" t="s">
-        <v>134</v>
+      <c r="O7" s="10" t="s">
+        <v>52</v>
       </c>
       <c r="P7" s="3"/>
       <c r="Q7" s="11" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R7" s="6" t="s">
         <v>7</v>
@@ -2507,63 +2619,63 @@
       <c r="S7" s="3"/>
       <c r="T7" s="10"/>
       <c r="U7" s="3" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="V7" s="11" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="W7" s="3" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="X7" s="6" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="Y7" s="3"/>
       <c r="Z7" s="3"/>
       <c r="AA7" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="AB7" s="3" t="s">
-        <v>229</v>
+        <v>164</v>
+      </c>
+      <c r="AB7" s="2" t="s">
+        <v>230</v>
       </c>
       <c r="AC7" s="3" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="AD7" s="2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="AE7" s="3"/>
       <c r="AF7" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="AG7" s="6" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="AH7" s="11" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="AI7" s="13"/>
       <c r="AJ7" s="2" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="AK7" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="AL7" s="3"/>
       <c r="AM7" s="3"/>
       <c r="AN7" s="3" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="AO7" s="3" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="AP7" s="3"/>
       <c r="AQ7" s="2" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="AR7" s="3"/>
       <c r="AS7" s="3" t="s">
-        <v>376</v>
+        <v>372</v>
       </c>
       <c r="AT7" s="3"/>
       <c r="AU7" s="3"/>
@@ -2578,90 +2690,90 @@
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
       <c r="F8" s="2" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="H8" s="2"/>
       <c r="I8" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
       <c r="L8" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="N8" s="2"/>
-      <c r="O8" s="10" t="s">
-        <v>53</v>
+      <c r="O8" s="11" t="s">
+        <v>185</v>
       </c>
       <c r="P8" s="2"/>
       <c r="Q8" s="10" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="R8" s="5" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="S8" s="2"/>
       <c r="T8" s="11"/>
       <c r="U8" s="2" t="s">
-        <v>357</v>
+        <v>353</v>
       </c>
       <c r="V8" s="10" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="W8" s="2" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="X8" s="5" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="Y8" s="2"/>
       <c r="Z8" s="2"/>
       <c r="AA8" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="AB8" s="2" t="s">
-        <v>234</v>
+        <v>179</v>
+      </c>
+      <c r="AB8" s="3" t="s">
+        <v>237</v>
       </c>
       <c r="AC8" s="2" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="AD8" s="3" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="AE8" s="2"/>
       <c r="AF8" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="AG8" s="5" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="AH8" s="10" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="AI8" s="12"/>
       <c r="AJ8" s="3" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="AK8" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="AL8" s="2"/>
       <c r="AM8" s="2"/>
       <c r="AN8" s="2" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="AO8" s="2" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="AP8" s="2"/>
       <c r="AQ8" s="3" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="AR8" s="2"/>
       <c r="AS8" s="2"/>
@@ -2679,81 +2791,81 @@
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
       <c r="G9" s="3" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="H9" s="3"/>
       <c r="I9" s="3" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
       <c r="L9" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="N9" s="3"/>
-      <c r="O9" s="11" t="s">
-        <v>187</v>
+      <c r="O9" s="10" t="s">
+        <v>197</v>
       </c>
       <c r="P9" s="3"/>
       <c r="Q9" s="11" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="R9" s="13"/>
       <c r="S9" s="3"/>
       <c r="T9" s="10"/>
       <c r="U9" s="3" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="V9" s="11" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="W9" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="X9" s="3"/>
       <c r="Y9" s="3"/>
       <c r="Z9" s="3"/>
       <c r="AA9" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="AB9" s="3" t="s">
-        <v>241</v>
+        <v>193</v>
+      </c>
+      <c r="AB9" s="2" t="s">
+        <v>242</v>
       </c>
       <c r="AC9" s="2" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="AD9" s="2" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="AE9" s="3"/>
       <c r="AF9" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="AG9" s="6" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="AH9" s="11" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="AI9" s="13"/>
       <c r="AJ9" s="3" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="AK9" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AL9" s="3"/>
       <c r="AM9" s="3"/>
       <c r="AN9" s="3"/>
       <c r="AO9" s="3" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="AP9" s="3"/>
       <c r="AQ9" s="2" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="AR9" s="3"/>
       <c r="AS9" s="3"/>
@@ -2771,21 +2883,21 @@
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
       <c r="G10" s="2" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
       <c r="L10" s="2" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="N10" s="2"/>
-      <c r="O10" s="10" t="s">
-        <v>199</v>
+      <c r="O10" s="11" t="s">
+        <v>207</v>
       </c>
       <c r="P10" s="2"/>
       <c r="Q10" s="10"/>
@@ -2793,51 +2905,49 @@
       <c r="S10" s="2"/>
       <c r="T10" s="11"/>
       <c r="U10" s="2" t="s">
-        <v>353</v>
+        <v>349</v>
       </c>
       <c r="V10" s="10" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="W10" s="2" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="X10" s="2"/>
       <c r="Y10" s="2"/>
       <c r="Z10" s="2"/>
       <c r="AA10" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="AB10" s="2" t="s">
-        <v>246</v>
-      </c>
+        <v>203</v>
+      </c>
+      <c r="AB10" s="2"/>
       <c r="AC10" s="2"/>
       <c r="AD10" s="3" t="s">
-        <v>372</v>
+        <v>368</v>
       </c>
       <c r="AE10" s="2"/>
       <c r="AF10" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="AG10" s="5" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="AH10" s="10" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="AI10" s="12"/>
       <c r="AJ10" s="2" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="AK10" s="2"/>
       <c r="AL10" s="2"/>
       <c r="AM10" s="2"/>
       <c r="AN10" s="2"/>
       <c r="AO10" s="2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="AP10" s="2"/>
       <c r="AQ10" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AR10" s="2"/>
       <c r="AS10" s="2"/>
@@ -2855,19 +2965,19 @@
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
       <c r="G11" s="3" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
       <c r="L11" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="M11" s="2"/>
       <c r="N11" s="3"/>
-      <c r="O11" s="11" t="s">
-        <v>209</v>
+      <c r="O11" s="10" t="s">
+        <v>256</v>
       </c>
       <c r="P11" s="3"/>
       <c r="Q11" s="3"/>
@@ -2875,47 +2985,47 @@
       <c r="S11" s="3"/>
       <c r="T11" s="3"/>
       <c r="U11" s="3" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="V11" s="11" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="W11" s="3" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="X11" s="3"/>
       <c r="Y11" s="3"/>
       <c r="Z11" s="3"/>
       <c r="AA11" s="3" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="AB11" s="3"/>
       <c r="AC11" s="3"/>
       <c r="AD11" s="2" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="AE11" s="3"/>
       <c r="AF11" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="AG11" s="6" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="AH11" s="3"/>
       <c r="AI11" s="3"/>
       <c r="AJ11" s="2" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="AK11" s="3"/>
       <c r="AL11" s="3"/>
       <c r="AM11" s="3"/>
       <c r="AN11" s="3"/>
       <c r="AO11" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="AP11" s="3"/>
       <c r="AQ11" s="3" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="AR11" s="3"/>
       <c r="AS11" s="3"/>
@@ -2933,49 +3043,47 @@
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
       <c r="G12" s="2" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="M12" s="2"/>
       <c r="N12" s="2"/>
-      <c r="O12" s="10" t="s">
-        <v>260</v>
-      </c>
+      <c r="O12" s="10"/>
       <c r="P12" s="2"/>
       <c r="Q12" s="2"/>
       <c r="R12" s="2"/>
       <c r="S12" s="2"/>
       <c r="T12" s="2"/>
       <c r="U12" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="V12" s="10" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="W12" s="2" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="X12" s="2"/>
       <c r="Y12" s="2"/>
       <c r="Z12" s="2"/>
       <c r="AA12" s="2" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
       <c r="AB12" s="2"/>
       <c r="AC12" s="2"/>
       <c r="AD12" s="3" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="AE12" s="2"/>
       <c r="AF12" s="2"/>
       <c r="AG12" s="5" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="AH12" s="2"/>
       <c r="AI12" s="2"/>
@@ -2985,11 +3093,11 @@
       <c r="AM12" s="2"/>
       <c r="AN12" s="2"/>
       <c r="AO12" s="2" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="AP12" s="2"/>
       <c r="AQ12" s="2" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="AR12" s="2"/>
       <c r="AS12" s="2"/>
@@ -3007,14 +3115,14 @@
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
       <c r="G13" s="3" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
       <c r="J13" s="3"/>
       <c r="K13" s="3"/>
       <c r="L13" s="3" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="M13" s="3"/>
       <c r="N13" s="3"/>
@@ -3025,24 +3133,24 @@
       <c r="S13" s="3"/>
       <c r="T13" s="3"/>
       <c r="U13" s="3" t="s">
-        <v>354</v>
+        <v>350</v>
       </c>
       <c r="V13" s="11" t="s">
-        <v>361</v>
+        <v>357</v>
       </c>
       <c r="W13" s="3" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="X13" s="3"/>
       <c r="Y13" s="3"/>
       <c r="Z13" s="3"/>
       <c r="AA13" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="AB13" s="3"/>
       <c r="AC13" s="3"/>
       <c r="AD13" s="3" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="AE13" s="3"/>
       <c r="AF13" s="3"/>
@@ -3054,12 +3162,10 @@
       <c r="AL13" s="3"/>
       <c r="AM13" s="3"/>
       <c r="AN13" s="3"/>
-      <c r="AO13" s="3" t="s">
-        <v>230</v>
-      </c>
+      <c r="AO13" s="3"/>
       <c r="AP13" s="3"/>
       <c r="AQ13" s="3" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="AR13" s="3"/>
       <c r="AS13" s="3"/>
@@ -3091,13 +3197,13 @@
       <c r="S14" s="2"/>
       <c r="T14" s="2"/>
       <c r="U14" s="2" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="V14" s="10" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
       <c r="W14" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="X14" s="2"/>
       <c r="Y14" s="2"/>
@@ -3119,7 +3225,7 @@
       <c r="AO14" s="2"/>
       <c r="AP14" s="2"/>
       <c r="AQ14" s="2" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="AR14" s="2"/>
       <c r="AS14" s="2"/>
@@ -3152,10 +3258,10 @@
       <c r="T15" s="3"/>
       <c r="U15" s="3"/>
       <c r="V15" s="11" t="s">
-        <v>362</v>
+        <v>358</v>
       </c>
       <c r="W15" s="3" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="X15" s="3"/>
       <c r="Y15" s="3"/>
@@ -3177,7 +3283,7 @@
       <c r="AO15" s="3"/>
       <c r="AP15" s="3"/>
       <c r="AQ15" s="2" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="AR15" s="3"/>
       <c r="AS15" s="3"/>
@@ -3210,10 +3316,10 @@
       <c r="T16" s="2"/>
       <c r="U16" s="2"/>
       <c r="V16" s="10" t="s">
-        <v>363</v>
+        <v>359</v>
       </c>
       <c r="W16" s="2" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="X16" s="2"/>
       <c r="Y16" s="2"/>
@@ -3235,7 +3341,7 @@
       <c r="AO16" s="2"/>
       <c r="AP16" s="2"/>
       <c r="AQ16" s="3" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="AR16" s="2"/>
       <c r="AS16" s="2"/>
@@ -3268,10 +3374,10 @@
       <c r="T17" s="3"/>
       <c r="U17" s="3"/>
       <c r="V17" s="11" t="s">
-        <v>364</v>
+        <v>360</v>
       </c>
       <c r="W17" s="3" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="X17" s="3"/>
       <c r="Y17" s="3"/>
@@ -3293,7 +3399,7 @@
       <c r="AO17" s="3"/>
       <c r="AP17" s="3"/>
       <c r="AQ17" s="2" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="AR17" s="3"/>
       <c r="AS17" s="3"/>
@@ -3326,10 +3432,10 @@
       <c r="T18" s="2"/>
       <c r="U18" s="2"/>
       <c r="V18" s="10" t="s">
-        <v>365</v>
+        <v>361</v>
       </c>
       <c r="W18" s="2" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="X18" s="2"/>
       <c r="Y18" s="2"/>
@@ -3351,7 +3457,7 @@
       <c r="AO18" s="2"/>
       <c r="AP18" s="2"/>
       <c r="AQ18" s="3" t="s">
-        <v>282</v>
+        <v>239</v>
       </c>
       <c r="AR18" s="2"/>
       <c r="AS18" s="2"/>
@@ -3384,10 +3490,10 @@
       <c r="T19" s="3"/>
       <c r="U19" s="3"/>
       <c r="V19" s="11" t="s">
-        <v>366</v>
+        <v>362</v>
       </c>
       <c r="W19" s="6" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="X19" s="3"/>
       <c r="Y19" s="3"/>
@@ -3408,9 +3514,7 @@
       <c r="AN19" s="3"/>
       <c r="AO19" s="3"/>
       <c r="AP19" s="3"/>
-      <c r="AQ19" s="3" t="s">
-        <v>243</v>
-      </c>
+      <c r="AQ19" s="3"/>
       <c r="AR19" s="3"/>
       <c r="AS19" s="3"/>
       <c r="AT19" s="3"/>
@@ -3442,10 +3546,10 @@
       <c r="T20" s="2"/>
       <c r="U20" s="2"/>
       <c r="V20" s="10" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="W20" s="5" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="X20" s="2"/>
       <c r="Y20" s="2"/>
@@ -3498,10 +3602,10 @@
       <c r="T21" s="3"/>
       <c r="U21" s="3"/>
       <c r="V21" s="11" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="W21" s="6" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="X21" s="3"/>
       <c r="Y21" s="3"/>
@@ -3554,10 +3658,10 @@
       <c r="T22" s="2"/>
       <c r="U22" s="2"/>
       <c r="V22" s="10" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="W22" s="5" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="X22" s="2"/>
       <c r="Y22" s="2"/>
@@ -3610,10 +3714,10 @@
       <c r="T23" s="3"/>
       <c r="U23" s="3"/>
       <c r="V23" s="11" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="W23" s="6" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="X23" s="3"/>
       <c r="Y23" s="3"/>
@@ -3667,7 +3771,7 @@
       <c r="U24" s="2"/>
       <c r="V24" s="2"/>
       <c r="W24" s="5" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="X24" s="2"/>
       <c r="Y24" s="2"/>
@@ -3699,22 +3803,22 @@
     </row>
     <row r="25" spans="1:50" x14ac:dyDescent="0.2">
       <c r="W25" s="6" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
     </row>
     <row r="26" spans="1:50" x14ac:dyDescent="0.2">
       <c r="W26" s="5" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
     </row>
     <row r="27" spans="1:50" x14ac:dyDescent="0.2">
       <c r="W27" s="6" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
     </row>
     <row r="28" spans="1:50" x14ac:dyDescent="0.2">
       <c r="W28" s="5" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
     </row>
   </sheetData>

</xml_diff>